<commit_message>
Rework ELC J-SOX controls and evidence
</commit_message>
<xml_diff>
--- a/4.evidence/ELC/内部通報受付台帳_FY2025.xlsx
+++ b/4.evidence/ELC/内部通報受付台帳_FY2025.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="内部通報受付台帳" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhistleblowingLog" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,11 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
-  </numFmts>
-  <fonts count="6">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,27 +27,12 @@
     </font>
     <font>
       <name val="Yu Gothic"/>
-      <b val="1"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Yu Gothic"/>
-      <i val="1"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Yu Gothic"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Yu Gothic"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -77,39 +59,30 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00888888"/>
+        <color rgb="00B7B7B7"/>
       </left>
       <right style="thin">
-        <color rgb="00888888"/>
+        <color rgb="00B7B7B7"/>
       </right>
       <top style="thin">
-        <color rgb="00888888"/>
+        <color rgb="00B7B7B7"/>
       </top>
       <bottom style="thin">
-        <color rgb="00888888"/>
+        <color rgb="00B7B7B7"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,113 +448,178 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【ELC-008 統制実施記録】 FY2025 内部通報受付台帳</t>
+          <t>通報番号</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>受付日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>受付ルート</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>概要</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>利益相反確認</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>調査責任者</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>財務報告影響評価</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>調査結果</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>是正/周知</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>監査等委員会報告日</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>完了日</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ステータス</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>管理者: 前田 美香（総務部長 GA001）/ 守秘義務あり（関係者限定閲覧）</t>
+          <t>WB-2025-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2025-07-15</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>外部弁護士</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>特定取引先への過剰接待疑い</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>総務部長に利害関係なし</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>総務部長 / 外部弁護士</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>直接影響なし。購買不正兆候なし。</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>接待規程の範囲内。ただし記録の粒度不足を確認。</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>接待申請時の相手先・目的記載を再周知</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-25</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>完了</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>通報番号</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>受付日</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>受付ルート</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>通報内容(要約)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>調査開始</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>調査結果</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>完了日</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>WB-2025-001</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>45853</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>外部弁護士経由</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>特定の取引先への過剰接待疑い（匿名）</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>45858</v>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>事実を確認、接待規程の範囲内と判断。注意喚起にとどめる。</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>45899</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>FY2025 受付件数: 1件 / 全件調査完了 / 監査等委員会報告済（2025/9/25）</t>
-        </is>
-      </c>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FY2025合計</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>受付1件、全件調査完了</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>財務報告へ直接影響する案件なし</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>監査等委員会へ四半期報告済</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>